<commit_message>
feat(knowledge_base): add REG-010 Client-Centricity regulation, card and update registries
</commit_message>
<xml_diff>
--- a/knowledge_base/00_РЕЕСТР/reestr-reglamentov.xlsx
+++ b/knowledge_base/00_РЕЕСТР/reestr-reglamentov.xlsx
@@ -115,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -145,6 +145,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -511,14 +514,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="53" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="49" customWidth="1" min="4" max="4"/>
-    <col width="86" customWidth="1" min="5" max="5"/>
+    <col width="88" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -852,6 +855,38 @@
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Утвержден</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>РЕГ-010</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Клиентоориентированность (внутренняя и внешняя)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Базовое Ядро</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Коммерческий директор / Собственник</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>Высокий уровень лояльности внешних клиентов и бесшовное взаимодействие подразделений</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>Утвержден</t>
         </is>
@@ -891,7 +926,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -1058,7 +1092,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(knowledge_base): remove REG-010 from approved registry, re-process as codified draft v0.1 in drafts/
</commit_message>
<xml_diff>
--- a/knowledge_base/00_РЕЕСТР/reestr-reglamentov.xlsx
+++ b/knowledge_base/00_РЕЕСТР/reestr-reglamentov.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -539,7 +539,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -855,38 +854,6 @@
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Утвержден</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>РЕГ-010</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>Клиентоориентированность (внутренняя и внешняя)</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Базовое Ядро</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>Коммерческий директор / Собственник</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>Высокий уровень лояльности внешних клиентов и бесшовное взаимодействие подразделений</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>Утвержден</t>
         </is>

</xml_diff>

<commit_message>
feat(knowledge_base): finalize REG-010 Client-Centricity as approved v1.0, update registries, record cumulative core rule (ADR-010)
</commit_message>
<xml_diff>
--- a/knowledge_base/00_РЕЕСТР/reestr-reglamentov.xlsx
+++ b/knowledge_base/00_РЕЕСТР/reestr-reglamentov.xlsx
@@ -514,14 +514,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="53" customWidth="1" min="2" max="2"/>
+    <col width="57" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="49" customWidth="1" min="4" max="4"/>
-    <col width="88" customWidth="1" min="5" max="5"/>
+    <col width="86" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -539,6 +539,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -854,6 +855,38 @@
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Утвержден</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>РЕГ-010</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Стандарт клиентоориентированности и клиентского опыта</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Базовое Ядро</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Коммерческий директор / HRD</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>Индекс лояльности NPS &gt;= 80%, повторные сделки &gt;= 20%, закрытие жалоб &lt;= 24 ч</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>Утвержден</t>
         </is>

</xml_diff>

<commit_message>
feat(knowledge_base): establish two-tier workflow folders (01_WORK_STAGING vs 02_CEO_APPROVED), update registries and decisions (ADR-011)
</commit_message>
<xml_diff>
--- a/knowledge_base/00_РЕЕСТР/reestr-reglamentov.xlsx
+++ b/knowledge_base/00_РЕЕСТР/reestr-reglamentov.xlsx
@@ -51,7 +51,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -88,6 +88,12 @@
         <bgColor rgb="00059669"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -115,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -147,6 +153,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -520,9 +538,9 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="57" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="49" customWidth="1" min="4" max="4"/>
-    <col width="86" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -535,7 +553,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Утвержденная нормативная база пилотного контура (v1.0) | Дата: Август 2026</t>
+          <t>Папка 1: Рабочий контур и согласование | Папка 2: Утверждено Генеральным директором</t>
         </is>
       </c>
     </row>
@@ -558,17 +576,17 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Владелец процесса (по Оргструктуре)</t>
+          <t>Владелец процесса</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Ценный конечный продукт (ЦКП)</t>
+          <t>Статус утверждения</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Статус</t>
+          <t>Размещение в базе</t>
         </is>
       </c>
     </row>
@@ -578,7 +596,7 @@
           <t>РЕГ-001</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Кодекс группы компаний Star Building</t>
         </is>
@@ -588,19 +606,19 @@
           <t>Базовое Ядро</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Собственник / Генеральный директор (CEO)</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Безопасность людей, качество конструкций, отсутствие фальсификаций</t>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Собственник / CEO</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Утвержден Гендиректором</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Утвержден</t>
+          <t>Папка 1 + Папка 2</t>
         </is>
       </c>
     </row>
@@ -610,9 +628,9 @@
           <t>РЕГ-002</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Общая оргструктура и штатная модель компании</t>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Общая оргструктура и штатная модель</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -620,19 +638,19 @@
           <t>Базовое Ядро</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Директор по персоналу (HRD) / CEO</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Иерархия подчинения, прозрачные зоны ответственности, исключение двоевластия</t>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Утвержден Гендиректором</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Утвержден</t>
+          <t>Папка 1 + Папка 2</t>
         </is>
       </c>
     </row>
@@ -642,7 +660,7 @@
           <t>РЕГ-003</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Стратегическая основа компании</t>
         </is>
@@ -652,19 +670,19 @@
           <t>Базовое Ядро</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Собственник / Генеральный директор (CEO)</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Генеральная цель, стратегия развития и ориентиры роста до 2030 года</t>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Собственник / CEO</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Утвержден Гендиректором</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Утвержден</t>
+          <t>Папка 1 + Папка 2</t>
         </is>
       </c>
     </row>
@@ -674,7 +692,7 @@
           <t>РЕГ-004</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Регламент «Как написать регламент»</t>
         </is>
@@ -684,19 +702,19 @@
           <t>Методологический</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>Методолог / Операционный директор (COO)</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>Единый корпоративный стандарт структуры и согласования регламентов</t>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Методолог / COO</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Утвержден Гендиректором</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Утвержден</t>
+          <t>Папка 1 + Папка 2</t>
         </is>
       </c>
     </row>
@@ -706,7 +724,7 @@
           <t>РЕГ-005</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Виды регламентов и их роль в компании</t>
         </is>
@@ -716,19 +734,19 @@
           <t>Методологический</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>Операционный директор (COO)</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>Иерархия нормативных документов компании (РГВ, операционные, карты)</t>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Утвержден Гендиректором</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>Утвержден</t>
+          <t>Папка 1 + Папка 2</t>
         </is>
       </c>
     </row>
@@ -738,7 +756,7 @@
           <t>РЕГ-006</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Правила ведения договорной работы</t>
         </is>
@@ -748,19 +766,19 @@
           <t>Операционный</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>Главный юрисконсульт / Правовой департамент</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>100% договоров проверены и подписаны без юридических и налоговых рисков</t>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Главный юрисконсульт / Правовой блок</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Утвержден Гендиректором</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Утвержден</t>
+          <t>Папка 1 + Папка 2</t>
         </is>
       </c>
     </row>
@@ -770,7 +788,7 @@
           <t>РЕГ-007</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>Кадровое делопроизводство</t>
         </is>
@@ -780,19 +798,19 @@
           <t>Операционный</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Директор по персоналу (HRD) / Кадровая служба</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>Своевременное документальное оформление приемов, отпусков, переводов, командировок</t>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>Директор по персоналу (HRD)</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Утвержден Гендиректором</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>Утвержден</t>
+          <t>Папка 1 + Папка 2</t>
         </is>
       </c>
     </row>
@@ -802,9 +820,9 @@
           <t>РЕГ-008</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Единая система мотивации, поощрения и выслуги лет</t>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Единая система мотивации, поощрения и выслуги</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -812,19 +830,19 @@
           <t>Операционный</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>Директор по персоналу (HRD) / CFO</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>Прозрачный расчет и выплата бонусной части, надбавок за стаж и выслугу</t>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Утвержден Гендиректором</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Утвержден</t>
+          <t>Папка 1 + Папка 2</t>
         </is>
       </c>
     </row>
@@ -834,7 +852,7 @@
           <t>РЕГ-009</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>Порядок выдачи и использования топливных карт</t>
         </is>
@@ -844,51 +862,51 @@
           <t>Операционный</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>Руководитель отдела логистики / Supply Chain</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>100% целевое использование корпоративных ГСМ, контроль лимитов</t>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Руководитель Supply Chain</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Утвержден Гендиректором</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>Утвержден</t>
+          <t>Папка 1 + Папка 2</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>РЕГ-010</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>Стандарт клиентоориентированности и клиентского опыта</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>Базовое Ядро</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
         <is>
           <t>Коммерческий директор / HRD</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>Индекс лояльности NPS &gt;= 80%, повторные сделки &gt;= 20%, закрытие жалоб &lt;= 24 ч</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Утвержден</t>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>На согласовании рабочей группой</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>Только Папка 1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor(knowledge_base): rename workflow directories to 01_В_РАБОТЕ and 02_УТВЕРЖДЕНО, update registries
</commit_message>
<xml_diff>
--- a/knowledge_base/00_РЕЕСТР/reestr-reglamentov.xlsx
+++ b/knowledge_base/00_РЕЕСТР/reestr-reglamentov.xlsx
@@ -540,7 +540,7 @@
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="35" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="31" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -553,7 +553,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Папка 1: Рабочий контур и согласование | Папка 2: Утверждено Генеральным директором</t>
+          <t>Папка 1: 01_В_РАБОТЕ (все + согласование) | Папка 2: 02_УТВЕРЖДЕНО (только Гендиректор)</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Папка 1 + Папка 2</t>
+          <t>01_В_РАБОТЕ + 02_УТВЕРЖДЕНО</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Папка 1 + Папка 2</t>
+          <t>01_В_РАБОТЕ + 02_УТВЕРЖДЕНО</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Папка 1 + Папка 2</t>
+          <t>01_В_РАБОТЕ + 02_УТВЕРЖДЕНО</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Папка 1 + Папка 2</t>
+          <t>01_В_РАБОТЕ + 02_УТВЕРЖДЕНО</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>Папка 1 + Папка 2</t>
+          <t>01_В_РАБОТЕ + 02_УТВЕРЖДЕНО</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Папка 1 + Папка 2</t>
+          <t>01_В_РАБОТЕ + 02_УТВЕРЖДЕНО</t>
         </is>
       </c>
     </row>
@@ -810,7 +810,7 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>Папка 1 + Папка 2</t>
+          <t>01_В_РАБОТЕ + 02_УТВЕРЖДЕНО</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Папка 1 + Папка 2</t>
+          <t>01_В_РАБОТЕ + 02_УТВЕРЖДЕНО</t>
         </is>
       </c>
     </row>
@@ -874,7 +874,7 @@
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>Папка 1 + Папка 2</t>
+          <t>01_В_РАБОТЕ + 02_УТВЕРЖДЕНО</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="F14" s="15" t="inlineStr">
         <is>
-          <t>Только Папка 1</t>
+          <t>Только 01_В_РАБОТЕ</t>
         </is>
       </c>
     </row>

</xml_diff>